<commit_message>
Actualizo por el archivo que he usado para crear gráficas
</commit_message>
<xml_diff>
--- a/resultados_experimentos/resumen_estadistico.xlsx
+++ b/resultados_experimentos/resumen_estadistico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universidadfv-my.sharepoint.com/personal/miguelangel_rojo_ufv_es/Documents/Escritorio/mike/Máster Inteligencia Artificial UPM/Sistemas Multiagente/Final Project/src/resultados_experimentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5A5DEB3-4BA2-4C3D-A1AF-BF5C642E190C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{A5A5DEB3-4BA2-4C3D-A1AF-BF5C642E190C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF03A620-DC99-4343-8194-F3372F122A78}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{94D7BA06-4934-4B9A-B985-571307B00BD3}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{94D7BA06-4934-4B9A-B985-571307B00BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="resumen_estadistico" sheetId="2" r:id="rId1"/>
@@ -149,9 +149,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -159,13 +158,7 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -192,7 +185,13 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -232,18 +231,18 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C2793F9-3C9C-4EB8-A7C1-EFFD448D93A8}" name="resumen_estadistico" displayName="resumen_estadistico" ref="A1:L13" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:L13" xr:uid="{8C2793F9-3C9C-4EB8-A7C1-EFFD448D93A8}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9D635FFA-3DC9-4BD8-B51E-C86AD5FDB374}" uniqueName="1" name="escenario" queryTableFieldId="1" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{93EDCE71-E4E8-46B1-BB0B-11A8D907FC85}" uniqueName="2" name="algoritmo" queryTableFieldId="2" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{F3A55797-9A03-4746-9C58-9207B883A984}" uniqueName="3" name="ejecuciones" queryTableFieldId="3" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{E8E85E63-257F-4AC8-90EE-5A07D00878E3}" uniqueName="4" name="media_distancia" queryTableFieldId="4" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{973AA077-8458-4607-85B1-11949C962452}" uniqueName="5" name="std_distancia" queryTableFieldId="5" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{7A23DD67-BE87-435C-84C6-78C293443CAD}" uniqueName="6" name="mediana_distancia" queryTableFieldId="6" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{BB1C4754-3E49-4BA0-9EED-33A5F0ADB87F}" uniqueName="7" name="mejor_distancia" queryTableFieldId="7" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{7901741F-8AD1-4280-A503-A7A420B18556}" uniqueName="8" name="peor_distancia" queryTableFieldId="8" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{887CFC56-1AD2-4DAF-9D82-9F6B63C4C02A}" uniqueName="9" name="media_tiempo" queryTableFieldId="9" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{B4B998B6-F5EB-40C4-911F-C0F53CCBC372}" uniqueName="10" name="std_tiempo" queryTableFieldId="10" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{DF306525-7860-4356-9DE1-05E766A1D0D9}" uniqueName="11" name="mediana_tiempo" queryTableFieldId="11" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{CA61CED8-FA15-47F3-8B74-2E47AB1F0A89}" uniqueName="12" name="cv_distancia" queryTableFieldId="12" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{9D635FFA-3DC9-4BD8-B51E-C86AD5FDB374}" uniqueName="1" name="escenario" queryTableFieldId="1" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{93EDCE71-E4E8-46B1-BB0B-11A8D907FC85}" uniqueName="2" name="algoritmo" queryTableFieldId="2" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F3A55797-9A03-4746-9C58-9207B883A984}" uniqueName="3" name="ejecuciones" queryTableFieldId="3" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E8E85E63-257F-4AC8-90EE-5A07D00878E3}" uniqueName="4" name="media_distancia" queryTableFieldId="4" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{973AA077-8458-4607-85B1-11949C962452}" uniqueName="5" name="std_distancia" queryTableFieldId="5" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{7A23DD67-BE87-435C-84C6-78C293443CAD}" uniqueName="6" name="mediana_distancia" queryTableFieldId="6" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{BB1C4754-3E49-4BA0-9EED-33A5F0ADB87F}" uniqueName="7" name="mejor_distancia" queryTableFieldId="7" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{7901741F-8AD1-4280-A503-A7A420B18556}" uniqueName="8" name="peor_distancia" queryTableFieldId="8" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{887CFC56-1AD2-4DAF-9D82-9F6B63C4C02A}" uniqueName="9" name="media_tiempo" queryTableFieldId="9" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{B4B998B6-F5EB-40C4-911F-C0F53CCBC372}" uniqueName="10" name="std_tiempo" queryTableFieldId="10" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{DF306525-7860-4356-9DE1-05E766A1D0D9}" uniqueName="11" name="mediana_tiempo" queryTableFieldId="11" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{CA61CED8-FA15-47F3-8B74-2E47AB1F0A89}" uniqueName="12" name="cv_distancia" queryTableFieldId="12" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -569,9 +568,9 @@
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.21875" bestFit="1" customWidth="1"/>
@@ -582,13 +581,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -620,458 +619,458 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2">
         <v>11.001175373295901</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2">
         <v>0.157462018436484</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2">
         <v>10.997122772037899</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>10.7463214546442</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2">
         <v>11.4078365117311</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2">
         <v>13.1811587266546</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2">
         <v>0.53074150268103004</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2">
         <v>13.1480078999884</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2">
         <v>1.43131995530864E-2</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>10.8186119902879</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>9.8438375841283995E-2</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>10.8225224241614</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>10.6382762491703</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3">
         <v>11.112893179059</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3">
         <v>40.933903496634798</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3">
         <v>1.6168647299897101</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3">
         <v>40.731867750058797</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3">
         <v>9.0989838557528693E-3</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>10.704712969685501</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>9.1447627643677407E-2</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>10.6996114253997</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>10.564119588583701</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4">
         <v>10.8993060812354</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4">
         <v>50.852171053333798</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4">
         <v>9.0901961627084997</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4">
         <v>53.189540149993199</v>
       </c>
-      <c r="L4" s="1">
+      <c r="L4">
         <v>8.5427444811127205E-3</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>11.0595822275926</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5">
         <v>0.16179369790241899</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5">
         <v>11.059552880004</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>10.703799836337501</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5">
         <v>11.3764525577425</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5">
         <v>41.094539923337202</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <v>1.1649651942786301</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5">
         <v>41.094021500088203</v>
       </c>
-      <c r="L5" s="1">
+      <c r="L5">
         <v>1.4629277541674099E-2</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6">
         <v>11.988681302840501</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6">
         <v>0.19084661405047901</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6">
         <v>12.011291796341499</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6">
         <v>11.544468242675</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6">
         <v>12.3540940508246</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6">
         <v>76.662825986688603</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6">
         <v>38.9667797857539</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6">
         <v>58.062092199921601</v>
       </c>
-      <c r="L6" s="1">
+      <c r="L6">
         <v>1.5918899604517901E-2</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7">
         <v>13.008797094349999</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7">
         <v>0.31844368798449202</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7">
         <v>13.0122182089835</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7">
         <v>12.531531270593399</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7">
         <v>13.6575831621885</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7">
         <v>3.86344773663828</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7">
         <v>0.715896936577056</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7">
         <v>4.0209912999998698</v>
       </c>
-      <c r="L7" s="1">
+      <c r="L7">
         <v>2.4479103307929798E-2</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8">
         <v>11.4924386044343</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8">
         <v>0.124358790463602</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8">
         <v>11.4653472080826</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8">
         <v>11.3358386158943</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8">
         <v>11.8641436696052</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8">
         <v>2.1674379800135801</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8">
         <v>8.3384802136822103E-2</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8">
         <v>2.1876212999923101</v>
       </c>
-      <c r="L8" s="1">
+      <c r="L8">
         <v>1.08209227600849E-2</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9">
         <v>11.328050804138099</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9">
         <v>5.5572932826894302E-2</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9">
         <v>11.3163339495658</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9">
         <v>11.221336245536801</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9">
         <v>11.4207586124539</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9">
         <v>85.045436163339701</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9">
         <v>7.9806030803837302</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9">
         <v>87.698279649950507</v>
       </c>
-      <c r="L9" s="1">
+      <c r="L9">
         <v>4.9057806844045298E-3</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10">
         <v>11.238037845989</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10">
         <v>3.58505882499916E-2</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <v>11.221336245536801</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10">
         <v>11.191517755389199</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10">
         <v>11.3630859404802</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10">
         <v>22.763165243357999</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10">
         <v>4.2444854725847998</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10">
         <v>21.5518790000351</v>
       </c>
-      <c r="L10" s="1">
+      <c r="L10">
         <v>3.1901110088169799E-3</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11">
         <v>11.4530917050937</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11">
         <v>0.152774804302752</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11">
         <v>11.4127965718507</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>11.275259576737801</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11">
         <v>11.880455166101401</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11">
         <v>25.8983280166673</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11">
         <v>14.535459834413301</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11">
         <v>22.431382750044499</v>
       </c>
-      <c r="L11" s="1">
+      <c r="L11">
         <v>1.33391758519497E-2</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>12.3866354840497</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12">
         <v>0.18366459089871601</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12">
         <v>12.382037088274901</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12">
         <v>11.8373142778873</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12">
         <v>12.697906278073701</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12">
         <v>28.560898393330401</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12">
         <v>7.5703661721379998</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12">
         <v>29.2417870500357</v>
       </c>
-      <c r="L12" s="1">
+      <c r="L12">
         <v>1.48276415444065E-2</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13">
         <v>13.4858493203918</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13">
         <v>0.45911197431869999</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13">
         <v>13.5617608614265</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13">
         <v>12.5282223075628</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13">
         <v>14.387866914272299</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13">
         <v>0.67506539671060894</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13">
         <v>2.3853628863216299E-2</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13">
         <v>0.67242235003504902</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13">
         <v>3.4043979241595197E-2</v>
       </c>
     </row>

</xml_diff>